<commit_message>
fix: keep demo workbook compatible with completed plans
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -1024,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1184,59 +1184,85 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>demo-b</v>
+        <v>demo-a</v>
       </c>
       <c r="B7" t="str">
-        <v>outsourcing</v>
+        <v>travel</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-09-30</v>
+        <v>2026-07-22</v>
       </c>
       <c r="D7" t="str">
-        <v>分析補助追加</v>
+        <v>共同研究旅費精算</v>
       </c>
       <c r="E7">
-        <v>90000</v>
+        <v>125000</v>
       </c>
       <c r="F7" t="str">
-        <v>demo-b-outsourcing-202609-001</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>追加解析のスポット対応分</v>
+        <v>計画額との差額55,000円を放棄して完了</v>
       </c>
       <c r="H7" t="str">
-        <v>要確認</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>demo-d</v>
+        <v>demo-b</v>
       </c>
       <c r="B8" t="str">
-        <v>low-balance</v>
+        <v>outsourcing</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-10-20</v>
+        <v>2026-09-30</v>
       </c>
       <c r="D8" t="str">
-        <v>年度末調整用消耗品</v>
+        <v>分析補助追加</v>
       </c>
       <c r="E8">
         <v>90000</v>
       </c>
       <c r="F8" t="str">
+        <v>demo-b-outsourcing-202609-001</v>
+      </c>
+      <c r="G8" t="str">
+        <v>追加解析のスポット対応分</v>
+      </c>
+      <c r="H8" t="str">
+        <v>要確認</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>demo-d</v>
+      </c>
+      <c r="B9" t="str">
+        <v>low-balance</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-10-20</v>
+      </c>
+      <c r="D9" t="str">
+        <v>年度末調整用消耗品</v>
+      </c>
+      <c r="E9">
+        <v>90000</v>
+      </c>
+      <c r="F9" t="str">
         <v>demo-d-low-balance-202610-001</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G9" t="str">
         <v>予定に紐づく一部執行</v>
       </c>
-      <c r="H8" t="str">
+      <c r="H9" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: extend demo seed across fiscal years
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,92 +457,144 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>demo-b</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B3" t="str">
-        <v>デモ研究費B</v>
+        <v>デモ研究費E（前年度）</v>
       </c>
       <c r="C3">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D3">
-        <v>800000</v>
+        <v>1200000</v>
       </c>
       <c r="E3" t="str">
-        <v>外注と解析補助が先行している比較用予算</v>
+        <v>前年度の執行結果を年度横断比較で確認するための予算</v>
       </c>
       <c r="F3" t="str">
-        <v>データ駆動解析</v>
+        <v/>
       </c>
       <c r="G3" t="str">
         <v/>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>demo-c</v>
+        <v>demo-f-next</v>
       </c>
       <c r="B4" t="str">
-        <v>デモ研究費C</v>
+        <v>デモ研究費F（翌年度）</v>
       </c>
       <c r="C4">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D4">
-        <v>500000</v>
+        <v>2000000</v>
       </c>
       <c r="E4" t="str">
-        <v>RA支出中心で変動の小さい比較用予算</v>
+        <v>翌年度の計画と先行手配を年度横断比較で確認するための予算</v>
       </c>
       <c r="F4" t="str">
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>学生支援</v>
+        <v/>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>demo-d</v>
+        <v>demo-b</v>
       </c>
       <c r="B5" t="str">
-        <v>デモ研究費D</v>
+        <v>デモ研究費B</v>
       </c>
       <c r="C5">
         <v>2026</v>
       </c>
       <c r="D5">
+        <v>800000</v>
+      </c>
+      <c r="E5" t="str">
+        <v>外注と解析補助が先行している比較用予算</v>
+      </c>
+      <c r="F5" t="str">
+        <v>データ駆動解析</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B6" t="str">
+        <v>デモ研究費C</v>
+      </c>
+      <c r="C6">
+        <v>2026</v>
+      </c>
+      <c r="D6">
         <v>500000</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E6" t="str">
+        <v>RA支出中心で変動の小さい比較用予算</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>学生支援</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>demo-d</v>
+      </c>
+      <c r="B7" t="str">
+        <v>デモ研究費D</v>
+      </c>
+      <c r="C7">
+        <v>2026</v>
+      </c>
+      <c r="D7">
+        <v>500000</v>
+      </c>
+      <c r="E7" t="str">
         <v>年度末に残高が少ない比較用予算</v>
       </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5">
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -614,16 +666,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>demo-b</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B5" t="str">
-        <v>outsourcing</v>
+        <v>legacy-equipment</v>
       </c>
       <c r="C5" t="str">
-        <v>委託費</v>
+        <v>物品費</v>
       </c>
       <c r="D5" t="str">
-        <v>other</v>
+        <v>equipment</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -631,10 +683,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>demo-c</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B6" t="str">
-        <v>personnel</v>
+        <v>legacy-personnel</v>
       </c>
       <c r="C6" t="str">
         <v>人件費</v>
@@ -643,36 +695,104 @@
         <v>personnel</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>demo-d</v>
+        <v>demo-f-next</v>
       </c>
       <c r="B7" t="str">
-        <v>low-balance</v>
+        <v>future-travel</v>
       </c>
       <c r="C7" t="str">
-        <v>低残高確認費</v>
+        <v>旅費</v>
       </c>
       <c r="D7" t="str">
-        <v>other</v>
+        <v>travel</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="B8" t="str">
+        <v>future-other</v>
+      </c>
+      <c r="C8" t="str">
+        <v>その他費</v>
+      </c>
+      <c r="D8" t="str">
+        <v>other</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>demo-b</v>
+      </c>
+      <c r="B9" t="str">
+        <v>outsourcing</v>
+      </c>
+      <c r="C9" t="str">
+        <v>委託費</v>
+      </c>
+      <c r="D9" t="str">
+        <v>other</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B10" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="C10" t="str">
+        <v>人件費</v>
+      </c>
+      <c r="D10" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>demo-d</v>
+      </c>
+      <c r="B11" t="str">
+        <v>low-balance</v>
+      </c>
+      <c r="C11" t="str">
+        <v>低残高確認費</v>
+      </c>
+      <c r="D11" t="str">
+        <v>other</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -732,56 +852,112 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>demo-b</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B5" t="str">
-        <v>outsourcing</v>
+        <v>legacy-equipment</v>
       </c>
       <c r="C5">
-        <v>500000</v>
+        <v>900000</v>
       </c>
       <c r="D5" t="str">
-        <v>解析支援の委託契約ベース</v>
+        <v>前年度に導入した計測・計算機器の予算枠</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>demo-c</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B6" t="str">
-        <v>personnel</v>
+        <v>legacy-personnel</v>
       </c>
       <c r="C6">
-        <v>240000</v>
+        <v>300000</v>
       </c>
       <c r="D6" t="str">
-        <v>被験者対応補助のRA謝金枠</v>
+        <v>前年度の研究補助者謝金枠</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="B7" t="str">
+        <v>future-travel</v>
+      </c>
+      <c r="C7">
+        <v>1200000</v>
+      </c>
+      <c r="D7" t="str">
+        <v>翌年度の国際会議・共同研究訪問の旅費枠</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="B8" t="str">
+        <v>future-other</v>
+      </c>
+      <c r="C8">
+        <v>800000</v>
+      </c>
+      <c r="D8" t="str">
+        <v>翌年度の共同研究基盤整備に備える枠</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>demo-b</v>
+      </c>
+      <c r="B9" t="str">
+        <v>outsourcing</v>
+      </c>
+      <c r="C9">
+        <v>500000</v>
+      </c>
+      <c r="D9" t="str">
+        <v>解析支援の委託契約ベース</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B10" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="C10">
+        <v>240000</v>
+      </c>
+      <c r="D10" t="str">
+        <v>被験者対応補助のRA謝金枠</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>demo-d</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B11" t="str">
         <v>low-balance</v>
       </c>
-      <c r="C7">
+      <c r="C11">
         <v>500000</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D11" t="str">
         <v>低残高リスクを確認するためのデモ枠</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1015,16 +1191,74 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>demo-f-travel-202705-001</v>
+      </c>
+      <c r="B9" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="C9" t="str">
+        <v>future-travel</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2027-05-12</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2027-05</v>
+      </c>
+      <c r="F9" t="str">
+        <v>国際共同研究旅費</v>
+      </c>
+      <c r="G9">
+        <v>720000</v>
+      </c>
+      <c r="H9" t="str">
+        <v>翌年度の国際共同研究と学会発表を想定</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>demo-f-other-202710-001</v>
+      </c>
+      <c r="B10" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="C10" t="str">
+        <v>future-other</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2027-10-01</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2027-10</v>
+      </c>
+      <c r="F10" t="str">
+        <v>共同研究基盤整備</v>
+      </c>
+      <c r="G10">
+        <v>400000</v>
+      </c>
+      <c r="H10" t="str">
+        <v>翌年度後半に予定する解析・共有基盤の整備</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1054,51 +1288,51 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>demo-a</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B2" t="str">
-        <v>travel</v>
+        <v>legacy-equipment</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-04-18</v>
+        <v>2025-07-25</v>
       </c>
       <c r="D2" t="str">
-        <v>研究会早割航空券</v>
+        <v>前年度計測機器更新</v>
       </c>
       <c r="E2">
-        <v>60000</v>
+        <v>560000</v>
       </c>
       <c r="F2" t="str">
-        <v>demo-a-travel-202607-001</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>発表参加に向けた早割手配</v>
+        <v>前年度の検収・支払済み金額</v>
       </c>
       <c r="H2" t="str">
-        <v>出張</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>demo-b</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B3" t="str">
-        <v>outsourcing</v>
+        <v>legacy-personnel</v>
       </c>
       <c r="C3" t="str">
-        <v>2026-04-28</v>
+        <v>2025-10-20</v>
       </c>
       <c r="D3" t="str">
-        <v>UI外注着手金</v>
+        <v>前年度RA謝金</v>
       </c>
       <c r="E3">
-        <v>410000</v>
+        <v>300000</v>
       </c>
       <c r="F3" t="str">
-        <v>demo-b-outsourcing-202604-001</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>初回納品分の検収後に計上</v>
+        <v>前年度後期分として支払済み</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -1109,48 +1343,48 @@
         <v>demo-a</v>
       </c>
       <c r="B4" t="str">
-        <v>equipment</v>
+        <v>travel</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-05-28</v>
+        <v>2026-04-18</v>
       </c>
       <c r="D4" t="str">
-        <v>GPUサーバ更新着手金</v>
+        <v>研究会早割航空券</v>
       </c>
       <c r="E4">
-        <v>300000</v>
+        <v>60000</v>
       </c>
       <c r="F4" t="str">
-        <v>demo-a-equipment-202605-001</v>
+        <v>demo-a-travel-202607-001</v>
       </c>
       <c r="G4" t="str">
-        <v>初回請求分、セットアップ作業を含む</v>
+        <v>発表参加に向けた早割手配</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>出張</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>demo-a</v>
+        <v>demo-b</v>
       </c>
       <c r="B5" t="str">
-        <v>supplies</v>
+        <v>outsourcing</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-06-12</v>
+        <v>2026-04-28</v>
       </c>
       <c r="D5" t="str">
-        <v>予備センサー購入</v>
+        <v>UI外注着手金</v>
       </c>
       <c r="E5">
-        <v>45000</v>
+        <v>410000</v>
       </c>
       <c r="F5" t="str">
-        <v>demo-a-supplies-202608-001</v>
+        <v>demo-b-outsourcing-202604-001</v>
       </c>
       <c r="G5" t="str">
-        <v>予備実験で追加購入した評価用センサー</v>
+        <v>初回納品分の検収後に計上</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -1158,25 +1392,25 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>demo-c</v>
+        <v>demo-a</v>
       </c>
       <c r="B6" t="str">
-        <v>personnel</v>
+        <v>equipment</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-06-25</v>
+        <v>2026-05-28</v>
       </c>
       <c r="D6" t="str">
-        <v>RA謝金</v>
+        <v>GPUサーバ更新着手金</v>
       </c>
       <c r="E6">
-        <v>90000</v>
+        <v>300000</v>
       </c>
       <c r="F6" t="str">
-        <v>demo-c-personnel-202606-001</v>
+        <v>demo-a-equipment-202605-001</v>
       </c>
       <c r="G6" t="str">
-        <v>実験補助RAの6月勤務分を計上</v>
+        <v>初回請求分、セットアップ作業を含む</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -1187,22 +1421,22 @@
         <v>demo-a</v>
       </c>
       <c r="B7" t="str">
-        <v>travel</v>
+        <v>supplies</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-07-22</v>
+        <v>2026-06-12</v>
       </c>
       <c r="D7" t="str">
-        <v>共同研究旅費精算</v>
+        <v>予備センサー購入</v>
       </c>
       <c r="E7">
-        <v>125000</v>
+        <v>45000</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>demo-a-supplies-202608-001</v>
       </c>
       <c r="G7" t="str">
-        <v>計画額との差額55,000円を放棄して完了</v>
+        <v>予備実験で追加購入した評価用センサー</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -1210,59 +1444,137 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>demo-b</v>
+        <v>demo-c</v>
       </c>
       <c r="B8" t="str">
-        <v>outsourcing</v>
+        <v>personnel</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-09-30</v>
+        <v>2026-06-25</v>
       </c>
       <c r="D8" t="str">
-        <v>分析補助追加</v>
+        <v>RA謝金</v>
       </c>
       <c r="E8">
         <v>90000</v>
       </c>
       <c r="F8" t="str">
-        <v>demo-b-outsourcing-202609-001</v>
+        <v>demo-c-personnel-202606-001</v>
       </c>
       <c r="G8" t="str">
-        <v>追加解析のスポット対応分</v>
+        <v>実験補助RAの6月勤務分を計上</v>
       </c>
       <c r="H8" t="str">
-        <v>要確認</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>demo-a</v>
+      </c>
+      <c r="B9" t="str">
+        <v>travel</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="D9" t="str">
+        <v>共同研究旅費精算</v>
+      </c>
+      <c r="E9">
+        <v>125000</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>計画額との差額55,000円を放棄して完了</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>demo-b</v>
+      </c>
+      <c r="B10" t="str">
+        <v>outsourcing</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="D10" t="str">
+        <v>分析補助追加</v>
+      </c>
+      <c r="E10">
+        <v>90000</v>
+      </c>
+      <c r="F10" t="str">
+        <v>demo-b-outsourcing-202609-001</v>
+      </c>
+      <c r="G10" t="str">
+        <v>追加解析のスポット対応分</v>
+      </c>
+      <c r="H10" t="str">
+        <v>要確認</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>demo-d</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B11" t="str">
         <v>low-balance</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C11" t="str">
         <v>2026-10-20</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D11" t="str">
         <v>年度末調整用消耗品</v>
       </c>
-      <c r="E9">
+      <c r="E11">
         <v>90000</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F11" t="str">
         <v>demo-d-low-balance-202610-001</v>
       </c>
-      <c r="G9" t="str">
+      <c r="G11" t="str">
         <v>予定に紐づく一部執行</v>
       </c>
-      <c r="H9" t="str">
+      <c r="H11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="B12" t="str">
+        <v>future-travel</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2027-05-25</v>
+      </c>
+      <c r="D12" t="str">
+        <v>国際共同研究旅費の先行手配</v>
+      </c>
+      <c r="E12">
+        <v>150000</v>
+      </c>
+      <c r="F12" t="str">
+        <v>demo-f-travel-202705-001</v>
+      </c>
+      <c r="G12" t="str">
+        <v>航空券と参加登録の先行支払分</v>
+      </c>
+      <c r="H12" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enrich cross-year demo edge cases
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -700,19 +700,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>demo-f-next</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B7" t="str">
-        <v>future-travel</v>
+        <v>legacy-reserve</v>
       </c>
       <c r="C7" t="str">
-        <v>旅費</v>
+        <v>予備費</v>
       </c>
       <c r="D7" t="str">
-        <v>travel</v>
+        <v>other</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -720,61 +720,61 @@
         <v>demo-f-next</v>
       </c>
       <c r="B8" t="str">
-        <v>future-other</v>
+        <v>future-travel</v>
       </c>
       <c r="C8" t="str">
-        <v>その他費</v>
+        <v>旅費</v>
       </c>
       <c r="D8" t="str">
-        <v>other</v>
+        <v>travel</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>demo-b</v>
+        <v>demo-f-next</v>
       </c>
       <c r="B9" t="str">
-        <v>outsourcing</v>
+        <v>future-other</v>
       </c>
       <c r="C9" t="str">
-        <v>委託費</v>
+        <v>その他費</v>
       </c>
       <c r="D9" t="str">
         <v>other</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>demo-c</v>
+        <v>demo-f-next</v>
       </c>
       <c r="B10" t="str">
-        <v>personnel</v>
+        <v>future-supplies</v>
       </c>
       <c r="C10" t="str">
-        <v>人件費</v>
+        <v>予備部材費</v>
       </c>
       <c r="D10" t="str">
-        <v>personnel</v>
+        <v>equipment</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>demo-d</v>
+        <v>demo-b</v>
       </c>
       <c r="B11" t="str">
-        <v>low-balance</v>
+        <v>outsourcing</v>
       </c>
       <c r="C11" t="str">
-        <v>低残高確認費</v>
+        <v>委託費</v>
       </c>
       <c r="D11" t="str">
         <v>other</v>
@@ -783,16 +783,50 @@
         <v>1</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B12" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="C12" t="str">
+        <v>人件費</v>
+      </c>
+      <c r="D12" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>demo-d</v>
+      </c>
+      <c r="B13" t="str">
+        <v>low-balance</v>
+      </c>
+      <c r="C13" t="str">
+        <v>低残高確認費</v>
+      </c>
+      <c r="D13" t="str">
+        <v>other</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -908,56 +942,70 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>demo-b</v>
+        <v>demo-f-next</v>
       </c>
       <c r="B9" t="str">
-        <v>outsourcing</v>
+        <v>future-supplies</v>
       </c>
       <c r="C9">
-        <v>500000</v>
+        <v>100000</v>
       </c>
       <c r="D9" t="str">
-        <v>解析支援の委託契約ベース</v>
+        <v>試作に必要な予備部材の小額枠</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>demo-c</v>
+        <v>demo-b</v>
       </c>
       <c r="B10" t="str">
-        <v>personnel</v>
+        <v>outsourcing</v>
       </c>
       <c r="C10">
-        <v>240000</v>
+        <v>500000</v>
       </c>
       <c r="D10" t="str">
-        <v>被験者対応補助のRA謝金枠</v>
+        <v>解析支援の委託契約ベース</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B11" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="C11">
+        <v>240000</v>
+      </c>
+      <c r="D11" t="str">
+        <v>被験者対応補助のRA謝金枠</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>demo-d</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>low-balance</v>
       </c>
-      <c r="C11">
+      <c r="C12">
         <v>500000</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D12" t="str">
         <v>低残高リスクを確認するためのデモ枠</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1249,16 +1297,45 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>demo-f-supplies-202802-001</v>
+      </c>
+      <c r="B11" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="C11" t="str">
+        <v>future-supplies</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2028-02-10</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2028-02</v>
+      </c>
+      <c r="F11" t="str">
+        <v>年度末試作部材</v>
+      </c>
+      <c r="G11">
+        <v>180000</v>
+      </c>
+      <c r="H11" t="str">
+        <v>費目枠を超えるが年度末の試作に必要な追加部材</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1297,16 +1374,16 @@
         <v>2025-07-25</v>
       </c>
       <c r="D2" t="str">
-        <v>前年度計測機器更新</v>
+        <v>前年度計測機器更新（中間支払）</v>
       </c>
       <c r="E2">
-        <v>560000</v>
+        <v>350000</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>前年度の検収・支払済み金額</v>
+        <v>前年度の検収後に支払った中間金</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -1317,22 +1394,22 @@
         <v>demo-e-legacy</v>
       </c>
       <c r="B3" t="str">
-        <v>legacy-personnel</v>
+        <v>legacy-equipment</v>
       </c>
       <c r="C3" t="str">
-        <v>2025-10-20</v>
+        <v>2025-08-20</v>
       </c>
       <c r="D3" t="str">
-        <v>前年度RA謝金</v>
+        <v>前年度計測機器更新（最終支払）</v>
       </c>
       <c r="E3">
-        <v>300000</v>
+        <v>210000</v>
       </c>
       <c r="F3" t="str">
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>前年度後期分として支払済み</v>
+        <v>検収後の最終支払分</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -1340,51 +1417,51 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>demo-a</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B4" t="str">
-        <v>travel</v>
+        <v>legacy-personnel</v>
       </c>
       <c r="C4" t="str">
-        <v>2026-04-18</v>
+        <v>2025-10-20</v>
       </c>
       <c r="D4" t="str">
-        <v>研究会早割航空券</v>
+        <v>前年度RA謝金</v>
       </c>
       <c r="E4">
-        <v>60000</v>
+        <v>300000</v>
       </c>
       <c r="F4" t="str">
-        <v>demo-a-travel-202607-001</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>発表参加に向けた早割手配</v>
+        <v>前年度後期分として支払済み</v>
       </c>
       <c r="H4" t="str">
-        <v>出張</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>demo-b</v>
+        <v>demo-e-legacy</v>
       </c>
       <c r="B5" t="str">
-        <v>outsourcing</v>
+        <v>legacy-reserve</v>
       </c>
       <c r="C5" t="str">
-        <v>2026-04-28</v>
+        <v>2026-03-18</v>
       </c>
       <c r="D5" t="str">
-        <v>UI外注着手金</v>
+        <v>前年度未予算調整</v>
       </c>
       <c r="E5">
-        <v>410000</v>
+        <v>50000</v>
       </c>
       <c r="F5" t="str">
-        <v>demo-b-outsourcing-202604-001</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>初回納品分の検収後に計上</v>
+        <v>年度末の未予算支出を精算</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -1395,48 +1472,48 @@
         <v>demo-a</v>
       </c>
       <c r="B6" t="str">
-        <v>equipment</v>
+        <v>travel</v>
       </c>
       <c r="C6" t="str">
-        <v>2026-05-28</v>
+        <v>2026-04-18</v>
       </c>
       <c r="D6" t="str">
-        <v>GPUサーバ更新着手金</v>
+        <v>研究会早割航空券</v>
       </c>
       <c r="E6">
-        <v>300000</v>
+        <v>60000</v>
       </c>
       <c r="F6" t="str">
-        <v>demo-a-equipment-202605-001</v>
+        <v>demo-a-travel-202607-001</v>
       </c>
       <c r="G6" t="str">
-        <v>初回請求分、セットアップ作業を含む</v>
+        <v>発表参加に向けた早割手配</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>出張</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>demo-a</v>
+        <v>demo-b</v>
       </c>
       <c r="B7" t="str">
-        <v>supplies</v>
+        <v>outsourcing</v>
       </c>
       <c r="C7" t="str">
-        <v>2026-06-12</v>
+        <v>2026-04-28</v>
       </c>
       <c r="D7" t="str">
-        <v>予備センサー購入</v>
+        <v>UI外注着手金</v>
       </c>
       <c r="E7">
-        <v>45000</v>
+        <v>410000</v>
       </c>
       <c r="F7" t="str">
-        <v>demo-a-supplies-202608-001</v>
+        <v>demo-b-outsourcing-202604-001</v>
       </c>
       <c r="G7" t="str">
-        <v>予備実験で追加購入した評価用センサー</v>
+        <v>初回納品分の検収後に計上</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -1444,25 +1521,25 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>demo-c</v>
+        <v>demo-a</v>
       </c>
       <c r="B8" t="str">
-        <v>personnel</v>
+        <v>equipment</v>
       </c>
       <c r="C8" t="str">
-        <v>2026-06-25</v>
+        <v>2026-05-28</v>
       </c>
       <c r="D8" t="str">
-        <v>RA謝金</v>
+        <v>GPUサーバ更新着手金</v>
       </c>
       <c r="E8">
-        <v>90000</v>
+        <v>300000</v>
       </c>
       <c r="F8" t="str">
-        <v>demo-c-personnel-202606-001</v>
+        <v>demo-a-equipment-202605-001</v>
       </c>
       <c r="G8" t="str">
-        <v>実験補助RAの6月勤務分を計上</v>
+        <v>初回請求分、セットアップ作業を含む</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -1473,22 +1550,22 @@
         <v>demo-a</v>
       </c>
       <c r="B9" t="str">
-        <v>travel</v>
+        <v>supplies</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-07-22</v>
+        <v>2026-06-12</v>
       </c>
       <c r="D9" t="str">
-        <v>共同研究旅費精算</v>
+        <v>予備センサー購入</v>
       </c>
       <c r="E9">
-        <v>125000</v>
+        <v>45000</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>demo-a-supplies-202608-001</v>
       </c>
       <c r="G9" t="str">
-        <v>計画額との差額55,000円を放棄して完了</v>
+        <v>予備実験で追加購入した評価用センサー</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -1496,51 +1573,51 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>demo-b</v>
+        <v>demo-c</v>
       </c>
       <c r="B10" t="str">
-        <v>outsourcing</v>
+        <v>personnel</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-09-30</v>
+        <v>2026-06-25</v>
       </c>
       <c r="D10" t="str">
-        <v>分析補助追加</v>
+        <v>RA謝金</v>
       </c>
       <c r="E10">
         <v>90000</v>
       </c>
       <c r="F10" t="str">
-        <v>demo-b-outsourcing-202609-001</v>
+        <v>demo-c-personnel-202606-001</v>
       </c>
       <c r="G10" t="str">
-        <v>追加解析のスポット対応分</v>
+        <v>実験補助RAの6月勤務分を計上</v>
       </c>
       <c r="H10" t="str">
-        <v>要確認</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>demo-d</v>
+        <v>demo-a</v>
       </c>
       <c r="B11" t="str">
-        <v>low-balance</v>
+        <v>travel</v>
       </c>
       <c r="C11" t="str">
-        <v>2026-10-20</v>
+        <v>2026-07-22</v>
       </c>
       <c r="D11" t="str">
-        <v>年度末調整用消耗品</v>
+        <v>共同研究旅費精算</v>
       </c>
       <c r="E11">
-        <v>90000</v>
+        <v>125000</v>
       </c>
       <c r="F11" t="str">
-        <v>demo-d-low-balance-202610-001</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>予定に紐づく一部執行</v>
+        <v>計画額との差額55,000円を放棄して完了</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -1548,33 +1625,111 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>demo-b</v>
+      </c>
+      <c r="B12" t="str">
+        <v>outsourcing</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="D12" t="str">
+        <v>分析補助追加</v>
+      </c>
+      <c r="E12">
+        <v>90000</v>
+      </c>
+      <c r="F12" t="str">
+        <v>demo-b-outsourcing-202609-001</v>
+      </c>
+      <c r="G12" t="str">
+        <v>追加解析のスポット対応分</v>
+      </c>
+      <c r="H12" t="str">
+        <v>要確認</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>demo-d</v>
+      </c>
+      <c r="B13" t="str">
+        <v>low-balance</v>
+      </c>
+      <c r="C13" t="str">
+        <v>2026-10-20</v>
+      </c>
+      <c r="D13" t="str">
+        <v>年度末調整用消耗品</v>
+      </c>
+      <c r="E13">
+        <v>90000</v>
+      </c>
+      <c r="F13" t="str">
+        <v>demo-d-low-balance-202610-001</v>
+      </c>
+      <c r="G13" t="str">
+        <v>予定に紐づく一部執行</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>demo-f-next</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B14" t="str">
         <v>future-travel</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C14" t="str">
         <v>2027-05-25</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D14" t="str">
         <v>国際共同研究旅費の先行手配</v>
       </c>
-      <c r="E12">
-        <v>150000</v>
-      </c>
-      <c r="F12" t="str">
+      <c r="E14">
+        <v>90000</v>
+      </c>
+      <c r="F14" t="str">
         <v>demo-f-travel-202705-001</v>
       </c>
-      <c r="G12" t="str">
-        <v>航空券と参加登録の先行支払分</v>
-      </c>
-      <c r="H12" t="str">
+      <c r="G14" t="str">
+        <v>航空券の先行支払分</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>demo-f-next</v>
+      </c>
+      <c r="B15" t="str">
+        <v>future-travel</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2027-06-30</v>
+      </c>
+      <c r="D15" t="str">
+        <v>国際共同研究旅費の追加精算</v>
+      </c>
+      <c r="E15">
+        <v>60000</v>
+      </c>
+      <c r="F15" t="str">
+        <v>demo-f-travel-202705-001</v>
+      </c>
+      <c r="G15" t="str">
+        <v>共同研究先訪問の追加精算分</v>
+      </c>
+      <c r="H15" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adjust future demo budget figures
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -492,7 +492,7 @@
         <v>2027</v>
       </c>
       <c r="D4">
-        <v>2000000</v>
+        <v>2200000</v>
       </c>
       <c r="E4" t="str">
         <v>翌年度の計画と先行手配を年度横断比較で確認するための予算</v>
@@ -948,7 +948,7 @@
         <v>future-supplies</v>
       </c>
       <c r="C9">
-        <v>100000</v>
+        <v>160000</v>
       </c>
       <c r="D9" t="str">
         <v>試作に必要な予備部材の小額枠</v>

</xml_diff>

<commit_message>
feat: add multiple demo funds per fiscal year
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -535,66 +535,118 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>demo-c</v>
+        <v>demo-g-legacy</v>
       </c>
       <c r="B6" t="str">
-        <v>デモ研究費C</v>
+        <v>デモ研究費G（前年度）</v>
       </c>
       <c r="C6">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D6">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="E6" t="str">
-        <v>RA支出中心で変動の小さい比較用予算</v>
+        <v>前年度に未執行で繰越判断を確認するための予算</v>
       </c>
       <c r="F6" t="str">
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>学生支援</v>
+        <v/>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>demo-h-next</v>
+      </c>
+      <c r="B7" t="str">
+        <v>デモ研究費H（翌年度）</v>
+      </c>
+      <c r="C7">
+        <v>2027</v>
+      </c>
+      <c r="D7">
+        <v>600000</v>
+      </c>
+      <c r="E7" t="str">
+        <v>翌年度の新規立ち上げ費を確認するための予算</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B8" t="str">
+        <v>デモ研究費C</v>
+      </c>
+      <c r="C8">
+        <v>2026</v>
+      </c>
+      <c r="D8">
+        <v>500000</v>
+      </c>
+      <c r="E8" t="str">
+        <v>RA支出中心で変動の小さい比較用予算</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>学生支援</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>demo-d</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B9" t="str">
         <v>デモ研究費D</v>
       </c>
-      <c r="C7">
+      <c r="C9">
         <v>2026</v>
       </c>
-      <c r="D7">
+      <c r="D9">
         <v>500000</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E9" t="str">
         <v>年度末に残高が少ない比較用予算</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7">
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -785,16 +837,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>demo-c</v>
+        <v>demo-g-legacy</v>
       </c>
       <c r="B12" t="str">
-        <v>personnel</v>
+        <v>legacy-travel</v>
       </c>
       <c r="C12" t="str">
-        <v>人件費</v>
+        <v>旅費</v>
       </c>
       <c r="D12" t="str">
-        <v>personnel</v>
+        <v>travel</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -802,31 +854,65 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>demo-d</v>
+        <v>demo-h-next</v>
       </c>
       <c r="B13" t="str">
-        <v>low-balance</v>
+        <v>future-personnel</v>
       </c>
       <c r="C13" t="str">
-        <v>低残高確認費</v>
+        <v>人件費</v>
       </c>
       <c r="D13" t="str">
-        <v>other</v>
+        <v>personnel</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B14" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="C14" t="str">
+        <v>人件費</v>
+      </c>
+      <c r="D14" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>demo-d</v>
+      </c>
+      <c r="B15" t="str">
+        <v>low-balance</v>
+      </c>
+      <c r="C15" t="str">
+        <v>低残高確認費</v>
+      </c>
+      <c r="D15" t="str">
+        <v>other</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -970,35 +1056,63 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>demo-c</v>
+        <v>demo-g-legacy</v>
       </c>
       <c r="B11" t="str">
-        <v>personnel</v>
+        <v>legacy-travel</v>
       </c>
       <c r="C11">
-        <v>240000</v>
+        <v>400000</v>
       </c>
       <c r="D11" t="str">
-        <v>被験者対応補助のRA謝金枠</v>
+        <v>前年度の未執行旅費枠</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>demo-h-next</v>
+      </c>
+      <c r="B12" t="str">
+        <v>future-personnel</v>
+      </c>
+      <c r="C12">
+        <v>600000</v>
+      </c>
+      <c r="D12" t="str">
+        <v>翌年度の新規立ち上げ人件費枠</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>demo-c</v>
+      </c>
+      <c r="B13" t="str">
+        <v>personnel</v>
+      </c>
+      <c r="C13">
+        <v>240000</v>
+      </c>
+      <c r="D13" t="str">
+        <v>被験者対応補助のRA謝金枠</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>demo-d</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B14" t="str">
         <v>low-balance</v>
       </c>
-      <c r="C12">
+      <c r="C14">
         <v>500000</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D14" t="str">
         <v>低残高リスクを確認するためのデモ枠</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: expose fiscal-year fund composition data
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -460,7 +460,7 @@
         <v>demo-e-legacy</v>
       </c>
       <c r="B3" t="str">
-        <v>デモ研究費E（前年度）</v>
+        <v>デモ継続研究費</v>
       </c>
       <c r="C3">
         <v>2025</v>
@@ -486,7 +486,7 @@
         <v>demo-f-next</v>
       </c>
       <c r="B4" t="str">
-        <v>デモ研究費F（翌年度）</v>
+        <v>デモ継続研究費</v>
       </c>
       <c r="C4">
         <v>2027</v>

</xml_diff>

<commit_message>
chore(demo): align recurring fund name across years
</commit_message>
<xml_diff>
--- a/seeds/demo/demo-budget.xlsx
+++ b/seeds/demo/demo-budget.xlsx
@@ -460,7 +460,7 @@
         <v>demo-e-legacy</v>
       </c>
       <c r="B3" t="str">
-        <v>デモ継続研究費</v>
+        <v>デモ研究費A</v>
       </c>
       <c r="C3">
         <v>2025</v>
@@ -486,7 +486,7 @@
         <v>demo-f-next</v>
       </c>
       <c r="B4" t="str">
-        <v>デモ継続研究費</v>
+        <v>デモ研究費A</v>
       </c>
       <c r="C4">
         <v>2027</v>

</xml_diff>